<commit_message>
Wed Aug  5 23:54:21 EEST 2026
</commit_message>
<xml_diff>
--- a/TLS_Germany/accounts.xlsx
+++ b/TLS_Germany/accounts.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="16">
   <si>
     <t>Account</t>
   </si>
@@ -43,7 +43,7 @@
     <t>Yallavisa@@123</t>
   </si>
   <si>
-    <t>August</t>
+    <t xml:space="preserve">October </t>
   </si>
   <si>
     <t xml:space="preserve">Alexandra </t>
@@ -56,6 +56,9 @@
   </si>
   <si>
     <t>tonil42212@rapplo.com</t>
+  </si>
+  <si>
+    <t>andrewyoussef2006@outlook.com</t>
   </si>
 </sst>
 </file>
@@ -505,18 +508,20 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="1"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
@@ -535,10 +540,10 @@
       <c r="Y5" s="2"/>
     </row>
     <row r="6">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
@@ -27372,33 +27377,6 @@
       <c r="X999" s="2"/>
       <c r="Y999" s="2"/>
     </row>
-    <row r="1000">
-      <c r="A1000" s="2"/>
-      <c r="B1000" s="2"/>
-      <c r="C1000" s="2"/>
-      <c r="D1000" s="2"/>
-      <c r="E1000" s="2"/>
-      <c r="F1000" s="2"/>
-      <c r="G1000" s="2"/>
-      <c r="H1000" s="2"/>
-      <c r="I1000" s="2"/>
-      <c r="J1000" s="2"/>
-      <c r="K1000" s="2"/>
-      <c r="L1000" s="2"/>
-      <c r="M1000" s="2"/>
-      <c r="N1000" s="2"/>
-      <c r="O1000" s="2"/>
-      <c r="P1000" s="2"/>
-      <c r="Q1000" s="2"/>
-      <c r="R1000" s="2"/>
-      <c r="S1000" s="2"/>
-      <c r="T1000" s="2"/>
-      <c r="U1000" s="2"/>
-      <c r="V1000" s="2"/>
-      <c r="W1000" s="2"/>
-      <c r="X1000" s="2"/>
-      <c r="Y1000" s="2"/>
-    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Sun Aug 30 19:15:38 EEST 2026
</commit_message>
<xml_diff>
--- a/TLS_Germany/accounts.xlsx
+++ b/TLS_Germany/accounts.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="19">
   <si>
     <t>Account</t>
   </si>
@@ -49,28 +49,25 @@
     <t>Alexandra</t>
   </si>
   <si>
+    <t>tonil42212@rapplo.com</t>
+  </si>
+  <si>
+    <t>andrewyoussef2006@outlook.com</t>
+  </si>
+  <si>
+    <t>yallavisa00@gmail.com</t>
+  </si>
+  <si>
+    <t>December</t>
+  </si>
+  <si>
+    <t>El-Sheikh Zayed</t>
+  </si>
+  <si>
     <t>mohamed71291@gmail.com</t>
   </si>
   <si>
     <t>moed-TLS-25</t>
-  </si>
-  <si>
-    <t>tonil42212@rapplo.com</t>
-  </si>
-  <si>
-    <t>andrewyoussef2006@outlook.com</t>
-  </si>
-  <si>
-    <t>yallavisa00@gmail.com</t>
-  </si>
-  <si>
-    <t>November</t>
-  </si>
-  <si>
-    <t>December</t>
-  </si>
-  <si>
-    <t>El-Sheikh Zayed</t>
   </si>
 </sst>
 </file>
@@ -407,13 +404,13 @@
         <v>12</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C3" s="2">
-        <v>57.0</v>
+        <v>58.0</v>
       </c>
       <c r="D3" s="2">
-        <v>120.0</v>
+        <v>200.0</v>
       </c>
       <c r="E3" s="5"/>
       <c r="F3" s="1" t="s">
@@ -428,17 +425,13 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="2">
-        <v>58.0</v>
-      </c>
-      <c r="D4" s="2">
-        <v>200.0</v>
-      </c>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
       <c r="E4" s="5"/>
       <c r="F4" s="1" t="s">
         <v>10</v>
@@ -452,66 +445,50 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
+      <c r="C5" s="2">
+        <v>3.0</v>
+      </c>
+      <c r="D5" s="2">
+        <v>200.0</v>
+      </c>
       <c r="E5" s="5"/>
       <c r="F5" s="1" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G5" s="2">
         <v>2026.0</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
+        <v>18</v>
+      </c>
+      <c r="C6" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="D6" s="2">
+        <v>120.0</v>
+      </c>
       <c r="E6" s="5"/>
       <c r="F6" s="1" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="G6" s="2">
         <v>2026.0</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>11</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" s="2">
-        <v>3.0</v>
-      </c>
-      <c r="D7" s="2">
-        <v>200.0</v>
-      </c>
-      <c r="E7" s="5"/>
-      <c r="F7" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="G7" s="2">
-        <v>2026.0</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>